<commit_message>
Remove hardcoded port 8502 from config.toml to fix Streamlit Cloud health check
</commit_message>
<xml_diff>
--- a/asistencias/historico_semanal.xlsx
+++ b/asistencias/historico_semanal.xlsx
@@ -103,31 +103,31 @@
     <t>19-jun-26</t>
   </si>
   <si>
-    <t>64.52% (20 de 31)</t>
-  </si>
-  <si>
-    <t>52.63% (20 de 38)</t>
-  </si>
-  <si>
-    <t>78.18% (43 de 55)</t>
-  </si>
-  <si>
-    <t>89.66% (52 de 58)</t>
-  </si>
-  <si>
-    <t>98.33% (59 de 60)</t>
-  </si>
-  <si>
-    <t>95.00% (57 de 60)</t>
-  </si>
-  <si>
-    <t>96.67% (58 de 60)</t>
-  </si>
-  <si>
-    <t>100.00% (12 de 12)</t>
-  </si>
-  <si>
-    <t>60.00% (12 de 20)</t>
+    <t>68.57% (24 de 35)</t>
+  </si>
+  <si>
+    <t>47.62% (20 de 42)</t>
+  </si>
+  <si>
+    <t>71.67% (43 de 60)</t>
+  </si>
+  <si>
+    <t>82.54% (52 de 63)</t>
+  </si>
+  <si>
+    <t>90.77% (59 de 65)</t>
+  </si>
+  <si>
+    <t>87.69% (57 de 65)</t>
+  </si>
+  <si>
+    <t>89.23% (58 de 65)</t>
+  </si>
+  <si>
+    <t>92.31% (12 de 13)</t>
+  </si>
+  <si>
+    <t>66.67% (16 de 24)</t>
   </si>
   <si>
     <t>80.00% (16 de 20)</t>
@@ -151,28 +151,28 @@
     <t>75.00% (9 de 12)</t>
   </si>
   <si>
-    <t>35.48% (11 de 31)</t>
-  </si>
-  <si>
-    <t>47.37% (18 de 38)</t>
-  </si>
-  <si>
-    <t>21.82% (12 de 55)</t>
-  </si>
-  <si>
-    <t>10.34% (6 de 58)</t>
-  </si>
-  <si>
-    <t>1.67% (1 de 60)</t>
-  </si>
-  <si>
-    <t>5.00% (3 de 60)</t>
-  </si>
-  <si>
-    <t>3.33% (2 de 60)</t>
-  </si>
-  <si>
-    <t>0.00% (0 de 12)</t>
+    <t>31.43% (11 de 35)</t>
+  </si>
+  <si>
+    <t>52.38% (22 de 42)</t>
+  </si>
+  <si>
+    <t>28.33% (17 de 60)</t>
+  </si>
+  <si>
+    <t>17.46% (11 de 63)</t>
+  </si>
+  <si>
+    <t>9.23% (6 de 65)</t>
+  </si>
+  <si>
+    <t>12.31% (8 de 65)</t>
+  </si>
+  <si>
+    <t>10.77% (7 de 65)</t>
+  </si>
+  <si>
+    <t>7.69% (1 de 13)</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
fix: Recalcular historico_semanal.xlsx con datos completos hasta semana 31 (27-31 Jul 2026)
</commit_message>
<xml_diff>
--- a/asistencias/historico_semanal.xlsx
+++ b/asistencias/historico_semanal.xlsx
@@ -14,11 +14,14 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="78">
   <si>
     <t>Semana</t>
   </si>
   <si>
+    <t>Año</t>
+  </si>
+  <si>
     <t>Fecha Inicio</t>
   </si>
   <si>
@@ -67,6 +70,12 @@
     <t>Semana 29</t>
   </si>
   <si>
+    <t>Semana 30</t>
+  </si>
+  <si>
+    <t>Semana 31</t>
+  </si>
+  <si>
     <t>05-may-26</t>
   </si>
   <si>
@@ -100,6 +109,12 @@
     <t>13-jul-26</t>
   </si>
   <si>
+    <t>20-jul-26</t>
+  </si>
+  <si>
+    <t>27-jul-26</t>
+  </si>
+  <si>
     <t>08-may-26</t>
   </si>
   <si>
@@ -130,13 +145,19 @@
     <t>10-jul-26</t>
   </si>
   <si>
-    <t>14-jul-26</t>
+    <t>17-jul-26</t>
+  </si>
+  <si>
+    <t>24-jul-26</t>
+  </si>
+  <si>
+    <t>31-jul-26</t>
   </si>
   <si>
     <t>68.57% (24 de 35)</t>
   </si>
   <si>
-    <t>47.62% (20 de 42)</t>
+    <t>48.39% (15 de 31)</t>
   </si>
   <si>
     <t>71.67% (43 de 60)</t>
@@ -160,13 +181,13 @@
     <t>87.69% (57 de 65)</t>
   </si>
   <si>
-    <t>88.46% (23 de 26)</t>
+    <t>86.15% (56 de 65)</t>
   </si>
   <si>
     <t>66.67% (16 de 24)</t>
   </si>
   <si>
-    <t>80.00% (16 de 20)</t>
+    <t>86.67% (13 de 15)</t>
   </si>
   <si>
     <t>65.12% (28 de 43)</t>
@@ -193,13 +214,16 @@
     <t>73.68% (42 de 57)</t>
   </si>
   <si>
-    <t>86.96% (20 de 23)</t>
+    <t>78.57% (44 de 56)</t>
+  </si>
+  <si>
+    <t>64.91% (37 de 57)</t>
   </si>
   <si>
     <t>31.43% (11 de 35)</t>
   </si>
   <si>
-    <t>52.38% (22 de 42)</t>
+    <t>51.61% (16 de 31)</t>
   </si>
   <si>
     <t>28.33% (17 de 60)</t>
@@ -223,7 +247,7 @@
     <t>12.31% (8 de 65)</t>
   </si>
   <si>
-    <t>11.54% (3 de 26)</t>
+    <t>13.85% (9 de 65)</t>
   </si>
 </sst>
 </file>
@@ -555,10 +579,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -577,225 +601,307 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>2026</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>33</v>
+      </c>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
+        <v>56</v>
+      </c>
+      <c r="G2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3">
+        <v>2026</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" t="s">
+        <v>47</v>
+      </c>
+      <c r="F3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G3" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4">
+        <v>2026</v>
+      </c>
+      <c r="C4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E4" t="s">
+        <v>48</v>
+      </c>
+      <c r="F4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G4" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>2026</v>
+      </c>
+      <c r="C5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6">
+        <v>2026</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G6" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7">
+        <v>2026</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F7" t="s">
+        <v>61</v>
+      </c>
+      <c r="G7" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8">
+        <v>2026</v>
+      </c>
+      <c r="C8" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" t="s">
+        <v>62</v>
+      </c>
+      <c r="G8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
+        <v>14</v>
+      </c>
+      <c r="B9">
+        <v>2026</v>
+      </c>
+      <c r="C9" t="s">
+        <v>27</v>
+      </c>
+      <c r="D9" t="s">
+        <v>40</v>
+      </c>
+      <c r="E9" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" t="s">
+        <v>63</v>
+      </c>
+      <c r="G9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10">
+        <v>2026</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G10" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
+        <v>16</v>
+      </c>
+      <c r="B11">
+        <v>2026</v>
+      </c>
+      <c r="C11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" t="s">
+        <v>65</v>
+      </c>
+      <c r="G11" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
         <v>17</v>
       </c>
-      <c r="C2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" t="s">
+      <c r="B12">
+        <v>2026</v>
+      </c>
+      <c r="C12" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D3" t="s">
-        <v>40</v>
-      </c>
-      <c r="E3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F3" t="s">
+      <c r="B13">
+        <v>2026</v>
+      </c>
+      <c r="C13" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" t="s">
+        <v>51</v>
+      </c>
+      <c r="F13" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="G13" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
         <v>19</v>
       </c>
-      <c r="C4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>51</v>
-      </c>
-      <c r="F4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" t="s">
-        <v>20</v>
-      </c>
-      <c r="C5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" t="s">
-        <v>42</v>
-      </c>
-      <c r="E5" t="s">
-        <v>52</v>
-      </c>
-      <c r="F5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B14">
+        <v>2026</v>
+      </c>
+      <c r="C14" t="s">
         <v>32</v>
       </c>
-      <c r="D6" t="s">
-        <v>43</v>
-      </c>
-      <c r="E6" t="s">
-        <v>53</v>
-      </c>
-      <c r="F6" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" t="s">
-        <v>33</v>
-      </c>
-      <c r="D7" t="s">
-        <v>44</v>
-      </c>
-      <c r="E7" t="s">
+      <c r="D14" t="s">
+        <v>45</v>
+      </c>
+      <c r="E14" t="s">
         <v>54</v>
       </c>
-      <c r="F7" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" t="s">
-        <v>55</v>
-      </c>
-      <c r="F8" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" t="s">
-        <v>35</v>
-      </c>
-      <c r="D9" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" t="s">
-        <v>57</v>
-      </c>
-      <c r="F10" t="s">
+      <c r="F14" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" t="s">
-        <v>58</v>
-      </c>
-      <c r="F11" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" t="s">
-        <v>27</v>
-      </c>
-      <c r="C12" t="s">
-        <v>38</v>
-      </c>
-      <c r="D12" t="s">
-        <v>48</v>
-      </c>
-      <c r="E12" t="s">
-        <v>59</v>
-      </c>
-      <c r="F12" t="s">
-        <v>69</v>
+      <c r="G14" t="s">
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>